<commit_message>
glass sound volume reduced from 300 to 10
</commit_message>
<xml_diff>
--- a/timekeeper.xlsx
+++ b/timekeeper.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G46"/>
+  <dimension ref="A1:G84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2057,6 +2057,1336 @@
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>NewTimekeeper</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>20260618-008</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>20.3</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>17:17:39</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>17:37:58</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>BMA_Prep4Consult</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>20260618-008</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>17:37:58</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>17:39:23</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>NewTimekeeper</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>20260618-008</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>17:39:23</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>17:47:39</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>NewTimekeeper</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>20260618-009</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>17:55:18</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>18:35:20</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>NewTimekeeper</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>20260618-010</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>70.90000000000001</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>18:35:36</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>19:46:30</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>NewTimekeeper</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>20260618-011</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>22:21:10</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>22:24:51</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>BMA_Prep4Consult</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>20260618-011</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>22:24:51</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>22:36:38</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>NewTimekeeper</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>20260618-011</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>22:36:38</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>22:51:10</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>NewTimekeeper</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>20260619-001</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>04:46:13</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>04:46:42</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>breakfast</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>20260619-001</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>04:46:42</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>04:52:55</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>NewTimekeeper</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>20260619-001</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>23.3</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>04:52:55</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>05:16:14</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>tautotita_mpampa</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>20260619-002</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="n">
+        <v>76.2</v>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>05:55:50</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>07:12:01</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>NewTimekeeper</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>20260619-003</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>5</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>07:57:10</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>08:02:13</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Climate_WP</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>20260619-003</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="n">
+        <v>85.7</v>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>08:02:13</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>09:27:56</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>ektypotis</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>20260619-004</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>09:36:24</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>10:11:41</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>ektypotis</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>20260619-005</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="n">
+        <v>32.2</v>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>10:12:10</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>10:44:24</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Αρχαγγελος</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>20260619-005</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>10:44:24</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>10:53:51</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Αρχαγγελος</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>20260619-006</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>10:54:05</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>11:24:05</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Αρχαγγελος</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>20260619-007</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>134.5</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>11:57:52</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>14:12:20</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>NewTimekeeper</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>20260619-007</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>14:12:20</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>14:18:17</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Climate_WP</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>20260619-007</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>13</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>14:18:17</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>14:31:16</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Climate_WP</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>20260619-008</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>14:39:36</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>15:20:15</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Climate_WP</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>20260619-009</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>17:21:41</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>17:33:34</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>NewTimekeeper</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>20260619-009</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="n">
+        <v>18.1</v>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>17:33:34</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>19:43:41</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>glyfada_ypogeio_lights</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>20260619-010</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>21:10:09</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>17:20:24</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>glyfada_υδραυλικά</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>20260620-001</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>17:37:03</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>18:07:03</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>cooking</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>20260620-002</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>18:20:33</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>18:28:23</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>NewTimekeeper</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>20260620-002</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>18:28:23</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>18:39:02</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>cooking</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>20260620-002</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>18:39:02</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>18:49:53</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>glyfada_υδραυλικά</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>20260620-002</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>18:49:53</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>18:50:33</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>zoi</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>20260620-003</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>18:57:36</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>19:18:21</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>friends</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>20260620-003</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>19:18:21</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>19:19:10</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>friends</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>20260620-004</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>30</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>19:43:53</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>20:13:53</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>aka8arista_giakopsimo</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>20260620-005</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>21:09:50</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>21:39:50</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>BMA_Prep4Consult</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>20260622-001</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>30</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>07:24:52</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>08:19:37</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>BMA_Prep4Consult</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>20260622-002</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>08:21:16</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>08:51:16</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>BMA_Prep4Consult</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>20260622-003</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>30</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>08:56:03</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>09:26:04</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>BMA_Prep4Consult</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>20260622-004</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>10:22:45</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>10:58:10</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>